<commit_message>
Removed (debug) code that is no longer needed in the long term. Updated tests. Updated documentation. Added a presentation.
</commit_message>
<xml_diff>
--- a/docs/Aufwands-SchaetzungUndErfassung_SignalReport.xlsx
+++ b/docs/Aufwands-SchaetzungUndErfassung_SignalReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\OneDrive\Programmieren\java_diplomlehrgang_2026_projekt\SignalReport\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{974A4DB0-8C8F-405E-87DD-47A1B21B41B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{932AE482-4A09-4955-A250-45807C3DF969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19830" yWindow="3120" windowWidth="32940" windowHeight="25530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3810" yWindow="1845" windowWidth="32940" windowHeight="25530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SignalReport" sheetId="1" r:id="rId1"/>
@@ -231,18 +231,12 @@
     <t>H2MeasurementRepositoryTest (10 Tests)</t>
   </si>
   <si>
-    <t>StatisticsTest (9 Tests)</t>
-  </si>
-  <si>
     <t>MeasurerInterfaceTest (6 Tests)</t>
   </si>
   <si>
     <t>MaintenanceWindowTest (7 Tests)</t>
   </si>
   <si>
-    <t>SessionManagerTest (16 Tests)</t>
-  </si>
-  <si>
     <t>Dokumentation</t>
   </si>
   <si>
@@ -391,6 +385,12 @@
   </si>
   <si>
     <t>Aufwandsschätzung und Dokumentation SignalReport</t>
+  </si>
+  <si>
+    <t>SessionManagerTest (19 Tests)</t>
+  </si>
+  <si>
+    <t>StatisticsTest (8 Tests)</t>
   </si>
 </sst>
 </file>
@@ -1030,7 +1030,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="42" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="L1" s="43" t="s">
         <v>0</v>
@@ -1780,7 +1780,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="54" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B57" s="55">
         <v>4</v>
@@ -1788,7 +1788,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="54" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B58" s="55">
         <v>2</v>
@@ -1846,7 +1846,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="54" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="B65" s="55">
         <v>1</v>
@@ -1854,7 +1854,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="54" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B66" s="55">
         <v>1</v>
@@ -1862,7 +1862,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="54" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B67" s="55">
         <v>1</v>
@@ -1870,7 +1870,7 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="54" t="s">
-        <v>66</v>
+        <v>115</v>
       </c>
       <c r="B68" s="55">
         <v>1.5</v>
@@ -1878,7 +1878,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B70" s="51"/>
       <c r="C70" s="52">
@@ -1896,7 +1896,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="54" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B71" s="55">
         <v>29</v>
@@ -1904,7 +1904,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="54" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B72" s="55">
         <v>5</v>
@@ -1912,7 +1912,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="54" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B73" s="55">
         <v>16</v>
@@ -1920,7 +1920,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="54" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B74" s="55">
         <v>8</v>
@@ -1928,7 +1928,7 @@
     </row>
     <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="60" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B77" s="61"/>
       <c r="C77" s="56">
@@ -1946,7 +1946,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B79" s="51"/>
       <c r="C79" s="51"/>
@@ -1955,7 +1955,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B80" s="55">
         <v>4.5</v>
@@ -1963,7 +1963,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B81" s="55">
         <v>3</v>
@@ -1971,7 +1971,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B82" s="55">
         <v>16</v>
@@ -1979,7 +1979,7 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="56" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B83" s="61"/>
       <c r="C83" s="56">
@@ -1991,7 +1991,7 @@
     </row>
     <row r="85" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A85" s="62" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B85" s="63"/>
       <c r="C85" s="64">
@@ -2003,7 +2003,7 @@
     </row>
     <row r="86" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A86" s="62" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B86" s="63"/>
       <c r="C86" s="65">
@@ -2041,10 +2041,10 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C1" s="66" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D1" s="67"/>
       <c r="E1" s="67"/>
@@ -2078,7 +2078,7 @@
         <v>11</v>
       </c>
       <c r="I3" s="66" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J3" s="67"/>
       <c r="K3" s="67"/>
@@ -2096,7 +2096,7 @@
         <v>0.2</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J4" t="s">
         <v>4</v>
@@ -2105,7 +2105,7 @@
         <v>5</v>
       </c>
       <c r="L4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="M4" t="s">
         <v>6</v>
@@ -2140,7 +2140,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="35">
@@ -2179,7 +2179,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="24" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B7" s="13">
         <v>6</v>
@@ -2214,7 +2214,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="24" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B8" s="13">
         <v>12</v>
@@ -2307,7 +2307,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="27">
@@ -2349,7 +2349,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="26" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B12" s="11">
         <v>4</v>
@@ -2384,7 +2384,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B13" s="11">
         <v>8</v>
@@ -2419,7 +2419,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B14" s="11">
         <v>32</v>
@@ -2474,7 +2474,7 @@
     </row>
     <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="23">
@@ -2490,7 +2490,7 @@
         <v>5.4</v>
       </c>
       <c r="K17" s="32" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="L17" s="32"/>
       <c r="M17" s="33">
@@ -2500,7 +2500,7 @@
     </row>
     <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="22" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B18" s="16">
         <v>6</v>
@@ -2509,7 +2509,7 @@
       <c r="D18" s="21"/>
       <c r="E18" s="21"/>
       <c r="K18" s="34" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L18" s="29"/>
       <c r="M18" s="30">
@@ -2519,7 +2519,7 @@
     </row>
     <row r="19" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B19" s="16">
         <v>4</v>
@@ -2532,7 +2532,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="22" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B20" s="16">
         <v>3</v>
@@ -2543,7 +2543,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B21" s="16">
         <v>2</v>
@@ -2554,7 +2554,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="22" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B22" s="16">
         <v>12</v>
@@ -2575,7 +2575,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="36">
@@ -2593,7 +2593,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B26" s="18">
         <v>4</v>
@@ -2604,7 +2604,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B27" s="18">
         <v>4</v>
@@ -2615,7 +2615,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B28" s="18">
         <v>4</v>
@@ -2637,7 +2637,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="35">
@@ -2655,7 +2655,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B32" s="13">
         <v>4</v>
@@ -2666,7 +2666,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="24" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B33" s="13">
         <v>2</v>
@@ -2677,7 +2677,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B34" s="13">
         <v>4</v>
@@ -2698,7 +2698,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B37" s="10"/>
       <c r="C37" s="27">
@@ -2716,7 +2716,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="26" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B38" s="11">
         <v>3</v>
@@ -2727,7 +2727,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="26" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B39" s="11">
         <v>6</v>
@@ -2738,7 +2738,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="26" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B40" s="11">
         <v>8</v>
@@ -2759,7 +2759,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B43" s="15"/>
       <c r="C43" s="23">
@@ -2777,7 +2777,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B44" s="16">
         <v>10</v>
@@ -2788,7 +2788,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="22" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B45" s="16">
         <v>12</v>
@@ -2799,7 +2799,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B46" s="16">
         <v>15</v>
@@ -2838,7 +2838,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B50" s="18">
         <v>12</v>
@@ -2849,7 +2849,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="25" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B51" s="18">
         <v>20</v>
@@ -2860,7 +2860,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="25" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B52" s="18">
         <v>30</v>
@@ -2878,7 +2878,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="12" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="35">
@@ -2895,7 +2895,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="24" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B56" s="13">
         <v>20</v>
@@ -2906,7 +2906,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="24" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B57" s="13">
         <v>10</v>
@@ -2917,7 +2917,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="24" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B58" s="13">
         <v>30</v>
@@ -2935,7 +2935,7 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B61" s="8"/>
       <c r="C61" s="20">
@@ -2953,7 +2953,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C63" s="7">
         <f>SUM(C61:E61)</f>

</xml_diff>

<commit_message>
Updating the database connection. Switching to a twin-DB architecture to improve crash resilience. Updating the documentation. Adapting the JUnit tests.
</commit_message>
<xml_diff>
--- a/docs/Aufwands-SchaetzungUndErfassung_SignalReport.xlsx
+++ b/docs/Aufwands-SchaetzungUndErfassung_SignalReport.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\OneDrive\Programmieren\java_diplomlehrgang_2026_projekt\SignalReport\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/601e3520dbede3a7/Programmieren/java_diplomlehrgang_2026_projekt/SignalReport/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{932AE482-4A09-4955-A250-45807C3DF969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{932AE482-4A09-4955-A250-45807C3DF969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EB8837A-8705-408E-A006-6581AC23ED2A}"/>
   <bookViews>
-    <workbookView xWindow="3810" yWindow="1845" windowWidth="32940" windowHeight="25530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11025" yWindow="975" windowWidth="32940" windowHeight="25530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SignalReport" sheetId="1" r:id="rId1"/>
@@ -668,7 +668,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -696,6 +695,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1014,9 +1016,9 @@
   <dimension ref="A1:M86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="1" max="1" width="37.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="3" customWidth="1"/>
@@ -1029,59 +1031,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="L1" s="43" t="s">
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="L1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="M1" s="44">
+      <c r="M1" s="43">
         <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="44" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="46"/>
-      <c r="B4" s="46" t="s">
+      <c r="A4" s="45"/>
+      <c r="B4" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="46" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="46" t="s">
+      <c r="C4" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="46" t="s">
+      <c r="E4" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="46" t="s">
+      <c r="H4" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="46" t="s">
+      <c r="I4" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="46" t="s">
+      <c r="J4" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="46" t="s">
+      <c r="K4" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="46" t="s">
+      <c r="L4" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="M4" s="46" t="s">
+      <c r="M4" s="45" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="D5" s="47" t="s">
+      <c r="D5" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="47" t="s">
+      <c r="E5" s="46" t="s">
         <v>11</v>
       </c>
       <c r="H5" t="str">
@@ -1104,16 +1110,16 @@
         <f t="shared" ref="L5:L13" si="0">SUM(I5:K5)</f>
         <v>82.5</v>
       </c>
-      <c r="M5" s="48">
+      <c r="M5" s="47">
         <f t="shared" ref="M5:M14" si="1">L5*$M$1</f>
         <v>4950</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="D6" s="49">
+      <c r="D6" s="48">
         <v>0.2</v>
       </c>
-      <c r="E6" s="49">
+      <c r="E6" s="48">
         <v>0.05</v>
       </c>
       <c r="H6" t="str">
@@ -1136,7 +1142,7 @@
         <f t="shared" si="0"/>
         <v>42.5</v>
       </c>
-      <c r="M6" s="48">
+      <c r="M6" s="47">
         <f t="shared" si="1"/>
         <v>2550</v>
       </c>
@@ -1162,25 +1168,25 @@
         <f t="shared" si="0"/>
         <v>77.5</v>
       </c>
-      <c r="M7" s="48">
+      <c r="M7" s="47">
         <f t="shared" si="1"/>
         <v>4650</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="51"/>
-      <c r="C8" s="52">
+      <c r="B8" s="50"/>
+      <c r="C8" s="51">
         <f>SUM(B9:B13)</f>
         <v>66</v>
       </c>
-      <c r="D8" s="53">
+      <c r="D8" s="52">
         <f>$C8*$D$6</f>
         <v>13.200000000000001</v>
       </c>
-      <c r="E8" s="53">
+      <c r="E8" s="52">
         <f>$C8*$E$6</f>
         <v>3.3000000000000003</v>
       </c>
@@ -1204,16 +1210,16 @@
         <f t="shared" si="0"/>
         <v>122.5</v>
       </c>
-      <c r="M8" s="48">
+      <c r="M8" s="47">
         <f t="shared" si="1"/>
         <v>7350</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="54" t="s">
+      <c r="A9" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="55">
+      <c r="B9" s="54">
         <v>8</v>
       </c>
       <c r="H9" t="str">
@@ -1236,16 +1242,16 @@
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
-      <c r="M9" s="48">
+      <c r="M9" s="47">
         <f t="shared" si="1"/>
         <v>3300</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="54" t="s">
+      <c r="A10" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="55">
+      <c r="B10" s="54">
         <v>8</v>
       </c>
       <c r="H10" t="str">
@@ -1268,16 +1274,16 @@
         <f t="shared" si="0"/>
         <v>52.5</v>
       </c>
-      <c r="M10" s="48">
+      <c r="M10" s="47">
         <f t="shared" si="1"/>
         <v>3150</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="54" t="s">
+      <c r="A11" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="55">
+      <c r="B11" s="54">
         <v>20</v>
       </c>
       <c r="H11" t="str">
@@ -1300,16 +1306,16 @@
         <f t="shared" si="0"/>
         <v>35.625</v>
       </c>
-      <c r="M11" s="48">
+      <c r="M11" s="47">
         <f t="shared" si="1"/>
         <v>2137.5</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="55">
+      <c r="B12" s="54">
         <v>16</v>
       </c>
       <c r="H12" t="str">
@@ -1332,16 +1338,16 @@
         <f t="shared" si="0"/>
         <v>11.25</v>
       </c>
-      <c r="M12" s="48">
+      <c r="M12" s="47">
         <f t="shared" si="1"/>
         <v>675</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="54" t="s">
+      <c r="A13" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="55">
+      <c r="B13" s="54">
         <v>14</v>
       </c>
       <c r="H13" t="str">
@@ -1364,7 +1370,7 @@
         <f t="shared" si="0"/>
         <v>72.5</v>
       </c>
-      <c r="M13" s="48">
+      <c r="M13" s="47">
         <f t="shared" si="1"/>
         <v>4350</v>
       </c>
@@ -1387,577 +1393,577 @@
         <f>I14</f>
         <v>23.5</v>
       </c>
-      <c r="M14" s="48">
+      <c r="M14" s="47">
         <f t="shared" si="1"/>
         <v>1410</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="51"/>
-      <c r="C15" s="52">
+      <c r="B15" s="50"/>
+      <c r="C15" s="51">
         <f>SUM(B16:B19)</f>
         <v>34</v>
       </c>
-      <c r="D15" s="53">
+      <c r="D15" s="52">
         <f>$C15*$D$6</f>
         <v>6.8000000000000007</v>
       </c>
-      <c r="E15" s="53">
+      <c r="E15" s="52">
         <f>$C15*$E$6</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="H15" s="56" t="s">
+      <c r="H15" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="56">
+      <c r="I15" s="55">
         <f>SUM(I5:I14)</f>
         <v>465</v>
       </c>
-      <c r="J15" s="56">
+      <c r="J15" s="55">
         <f>SUM(J5:J14)</f>
         <v>88.300000000000011</v>
       </c>
-      <c r="K15" s="56">
+      <c r="K15" s="55">
         <f>SUM(K5:K14)</f>
         <v>22.075000000000003</v>
       </c>
-      <c r="L15" s="57">
+      <c r="L15" s="56">
         <f>SUM(L5:L14)</f>
         <v>575.375</v>
       </c>
-      <c r="M15" s="58">
+      <c r="M15" s="57">
         <f>SUM(M5:M14)</f>
         <v>34522.5</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="54" t="s">
+      <c r="A16" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="55">
+      <c r="B16" s="54">
         <v>6</v>
       </c>
-      <c r="H16" s="47" t="s">
+      <c r="H16" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L16" s="59" t="str">
+      <c r="L16" s="58" t="str">
         <f>IF(L15=C85,"OK","FEHLER!")</f>
         <v>OK</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="54" t="s">
+      <c r="A17" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="55">
+      <c r="B17" s="54">
         <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="54" t="s">
+      <c r="A18" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="55">
+      <c r="B18" s="54">
         <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="54" t="s">
+      <c r="A19" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="55">
+      <c r="B19" s="54">
         <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="50" t="s">
+      <c r="A21" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="51"/>
-      <c r="C21" s="52">
+      <c r="B21" s="50"/>
+      <c r="C21" s="51">
         <f>SUM(B22:B27)</f>
         <v>62</v>
       </c>
-      <c r="D21" s="53">
+      <c r="D21" s="52">
         <f>$C21*$D$6</f>
         <v>12.4</v>
       </c>
-      <c r="E21" s="53">
+      <c r="E21" s="52">
         <f>$C21*$E$6</f>
         <v>3.1</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="55">
+      <c r="B22" s="54">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="54" t="s">
+      <c r="A23" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="55">
+      <c r="B23" s="54">
         <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="54" t="s">
+      <c r="A24" s="53" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="55">
+      <c r="B24" s="54">
         <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="54" t="s">
+      <c r="A25" s="53" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="55">
+      <c r="B25" s="54">
         <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="54" t="s">
+      <c r="A26" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="55">
+      <c r="B26" s="54">
         <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="54" t="s">
+      <c r="A27" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="55">
+      <c r="B27" s="54">
         <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="50" t="s">
+      <c r="A29" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="51"/>
-      <c r="C29" s="52">
+      <c r="B29" s="50"/>
+      <c r="C29" s="51">
         <f>SUM(B30:B36)</f>
         <v>98</v>
       </c>
-      <c r="D29" s="53">
+      <c r="D29" s="52">
         <f>$C29*$D$6</f>
         <v>19.600000000000001</v>
       </c>
-      <c r="E29" s="53">
+      <c r="E29" s="52">
         <f>$C29*$E$6</f>
         <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="54" t="s">
+      <c r="A30" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="55">
+      <c r="B30" s="54">
         <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="54" t="s">
+      <c r="A31" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="55">
+      <c r="B31" s="54">
         <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="54" t="s">
+      <c r="A32" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="55">
+      <c r="B32" s="54">
         <v>16</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="54" t="s">
+      <c r="A33" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="55">
+      <c r="B33" s="54">
         <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="54" t="s">
+      <c r="A34" s="53" t="s">
         <v>38</v>
       </c>
-      <c r="B34" s="55">
+      <c r="B34" s="54">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="54" t="s">
+      <c r="A35" s="53" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="55">
+      <c r="B35" s="54">
         <v>12</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="54" t="s">
+      <c r="A36" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="B36" s="55">
+      <c r="B36" s="54">
         <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="50" t="s">
+      <c r="A38" s="49" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="51"/>
-      <c r="C38" s="52">
+      <c r="B38" s="50"/>
+      <c r="C38" s="51">
         <f>SUM(B39:B44)</f>
         <v>44</v>
       </c>
-      <c r="D38" s="53">
+      <c r="D38" s="52">
         <f>$C38*$D$6</f>
         <v>8.8000000000000007</v>
       </c>
-      <c r="E38" s="53">
+      <c r="E38" s="52">
         <f>$C38*$E$6</f>
         <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="54" t="s">
+      <c r="A39" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="55">
+      <c r="B39" s="54">
         <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="54" t="s">
+      <c r="A40" s="53" t="s">
         <v>43</v>
       </c>
-      <c r="B40" s="55">
+      <c r="B40" s="54">
         <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="54" t="s">
+      <c r="A41" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="55">
+      <c r="B41" s="54">
         <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="54" t="s">
+      <c r="A42" s="53" t="s">
         <v>45</v>
       </c>
-      <c r="B42" s="55">
+      <c r="B42" s="54">
         <v>8</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="54" t="s">
+      <c r="A43" s="53" t="s">
         <v>46</v>
       </c>
-      <c r="B43" s="55">
+      <c r="B43" s="54">
         <v>8</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="54" t="s">
+      <c r="A44" s="53" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="55">
+      <c r="B44" s="54">
         <v>6</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="50" t="s">
+      <c r="A46" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="B46" s="51"/>
-      <c r="C46" s="52">
+      <c r="B46" s="50"/>
+      <c r="C46" s="51">
         <f>SUM(B47:B50)</f>
         <v>42</v>
       </c>
-      <c r="D46" s="53">
+      <c r="D46" s="52">
         <f>$C46*$D$6</f>
         <v>8.4</v>
       </c>
-      <c r="E46" s="53">
+      <c r="E46" s="52">
         <f>$C46*$E$6</f>
         <v>2.1</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="54" t="s">
+      <c r="A47" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="B47" s="55">
+      <c r="B47" s="54">
         <v>20</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="54" t="s">
+      <c r="A48" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="B48" s="55">
+      <c r="B48" s="54">
         <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="54" t="s">
+      <c r="A49" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="B49" s="55">
+      <c r="B49" s="54">
         <v>12</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="54" t="s">
+      <c r="A50" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="B50" s="55">
+      <c r="B50" s="54">
         <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="50" t="s">
+      <c r="A52" s="49" t="s">
         <v>53</v>
       </c>
-      <c r="B52" s="51"/>
-      <c r="C52" s="52">
+      <c r="B52" s="50"/>
+      <c r="C52" s="51">
         <f>SUM(B53:B58)</f>
         <v>28.5</v>
       </c>
-      <c r="D52" s="53">
+      <c r="D52" s="52">
         <f>$C52*$D$6</f>
         <v>5.7</v>
       </c>
-      <c r="E52" s="53">
+      <c r="E52" s="52">
         <f>$C52*$E$6</f>
         <v>1.425</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="54" t="s">
+      <c r="A53" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="B53" s="55">
+      <c r="B53" s="54">
         <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="54" t="s">
+      <c r="A54" s="53" t="s">
         <v>55</v>
       </c>
-      <c r="B54" s="55">
+      <c r="B54" s="54">
         <v>2.5</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="54" t="s">
+      <c r="A55" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B55" s="55">
+      <c r="B55" s="54">
         <v>10</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="54" t="s">
+      <c r="A56" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="B56" s="55">
+      <c r="B56" s="54">
         <v>6</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="54" t="s">
+      <c r="A57" s="53" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="55">
+      <c r="B57" s="54">
         <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="54" t="s">
+      <c r="A58" s="53" t="s">
         <v>113</v>
       </c>
-      <c r="B58" s="55">
+      <c r="B58" s="54">
         <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="50" t="s">
+      <c r="A60" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="51"/>
-      <c r="C60" s="52">
+      <c r="B60" s="50"/>
+      <c r="C60" s="51">
         <f>SUM(B61:B68)</f>
         <v>9</v>
       </c>
-      <c r="D60" s="53">
+      <c r="D60" s="52">
         <f>$C60*$D$6</f>
         <v>1.8</v>
       </c>
-      <c r="E60" s="53">
+      <c r="E60" s="52">
         <f>$C60*$E$6</f>
         <v>0.45</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="54" t="s">
+      <c r="A61" s="53" t="s">
         <v>59</v>
       </c>
-      <c r="B61" s="55">
+      <c r="B61" s="54">
         <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="54" t="s">
+      <c r="A62" s="53" t="s">
         <v>60</v>
       </c>
-      <c r="B62" s="55">
+      <c r="B62" s="54">
         <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="54" t="s">
+      <c r="A63" s="53" t="s">
         <v>61</v>
       </c>
-      <c r="B63" s="55">
+      <c r="B63" s="54">
         <v>1.5</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="54" t="s">
+      <c r="A64" s="53" t="s">
         <v>62</v>
       </c>
-      <c r="B64" s="55">
+      <c r="B64" s="54">
         <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="54" t="s">
+      <c r="A65" s="53" t="s">
         <v>116</v>
       </c>
-      <c r="B65" s="55">
+      <c r="B65" s="54">
         <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="54" t="s">
+      <c r="A66" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="B66" s="55">
+      <c r="B66" s="54">
         <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="54" t="s">
+      <c r="A67" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="55">
+      <c r="B67" s="54">
         <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="54" t="s">
+      <c r="A68" s="53" t="s">
         <v>115</v>
       </c>
-      <c r="B68" s="55">
+      <c r="B68" s="54">
         <v>1.5</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="50" t="s">
+      <c r="A70" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="B70" s="51"/>
-      <c r="C70" s="52">
+      <c r="B70" s="50"/>
+      <c r="C70" s="51">
         <f>SUM(B71:B74)</f>
         <v>58</v>
       </c>
-      <c r="D70" s="53">
+      <c r="D70" s="52">
         <f>$C70*$D$6</f>
         <v>11.600000000000001</v>
       </c>
-      <c r="E70" s="53">
+      <c r="E70" s="52">
         <f>$C70*$E$6</f>
         <v>2.9000000000000004</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="54" t="s">
+      <c r="A71" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="B71" s="55">
+      <c r="B71" s="54">
         <v>29</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="54" t="s">
+      <c r="A72" s="53" t="s">
         <v>67</v>
       </c>
-      <c r="B72" s="55">
+      <c r="B72" s="54">
         <v>5</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="54" t="s">
+      <c r="A73" s="53" t="s">
         <v>68</v>
       </c>
-      <c r="B73" s="55">
+      <c r="B73" s="54">
         <v>16</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="54" t="s">
+      <c r="A74" s="53" t="s">
         <v>69</v>
       </c>
-      <c r="B74" s="55">
+      <c r="B74" s="54">
         <v>8</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A77" s="60" t="s">
+      <c r="A77" s="59" t="s">
         <v>70</v>
       </c>
-      <c r="B77" s="61"/>
-      <c r="C77" s="56">
+      <c r="B77" s="60"/>
+      <c r="C77" s="55">
         <f>C8+C15+C21+C29+C38+C46+C52+C60+C70</f>
         <v>441.5</v>
       </c>
-      <c r="D77" s="57">
+      <c r="D77" s="56">
         <f>D8+D15+D21+D29+D38+D46+D52+D60+D70</f>
         <v>88.300000000000011</v>
       </c>
-      <c r="E77" s="57">
+      <c r="E77" s="56">
         <f>E8+E15+E21+E29+E38+E46+E52+E60+E70</f>
         <v>22.075000000000003</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="50" t="s">
+      <c r="A79" s="49" t="s">
         <v>71</v>
       </c>
-      <c r="B79" s="51"/>
-      <c r="C79" s="51"/>
-      <c r="D79" s="51"/>
-      <c r="E79" s="51"/>
+      <c r="B79" s="50"/>
+      <c r="C79" s="50"/>
+      <c r="D79" s="50"/>
+      <c r="E79" s="50"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>72</v>
       </c>
-      <c r="B80" s="55">
+      <c r="B80" s="54">
         <v>4.5</v>
       </c>
     </row>
@@ -1965,7 +1971,7 @@
       <c r="A81" t="s">
         <v>73</v>
       </c>
-      <c r="B81" s="55">
+      <c r="B81" s="54">
         <v>3</v>
       </c>
     </row>
@@ -1973,48 +1979,52 @@
       <c r="A82" t="s">
         <v>74</v>
       </c>
-      <c r="B82" s="55">
+      <c r="B82" s="54">
         <v>16</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="56" t="s">
+      <c r="A83" s="55" t="s">
         <v>75</v>
       </c>
-      <c r="B83" s="61"/>
-      <c r="C83" s="56">
+      <c r="B83" s="60"/>
+      <c r="C83" s="55">
         <f>SUM(B80:B82)</f>
         <v>23.5</v>
       </c>
-      <c r="D83" s="61"/>
-      <c r="E83" s="61"/>
+      <c r="D83" s="60"/>
+      <c r="E83" s="60"/>
     </row>
     <row r="85" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A85" s="62" t="s">
+      <c r="A85" s="61" t="s">
         <v>76</v>
       </c>
-      <c r="B85" s="63"/>
-      <c r="C85" s="64">
+      <c r="B85" s="62"/>
+      <c r="C85" s="63">
         <f>C77+D77+E77+C83</f>
         <v>575.375</v>
       </c>
-      <c r="D85" s="63"/>
-      <c r="E85" s="63"/>
+      <c r="D85" s="62"/>
+      <c r="E85" s="62"/>
     </row>
     <row r="86" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A86" s="62" t="s">
+      <c r="A86" s="61" t="s">
         <v>77</v>
       </c>
-      <c r="B86" s="63"/>
-      <c r="C86" s="65">
+      <c r="B86" s="62"/>
+      <c r="C86" s="64">
         <f>C85*$M$1</f>
         <v>34522.5</v>
       </c>
-      <c r="D86" s="63"/>
-      <c r="E86" s="63"/>
+      <c r="D86" s="62"/>
+      <c r="E86" s="62"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2043,11 +2053,11 @@
       <c r="B1" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="66" t="s">
+      <c r="C1" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
       <c r="L1" t="s">
         <v>0</v>
       </c>
@@ -2077,12 +2087,12 @@
       <c r="E3" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="66" t="s">
+      <c r="I3" s="65" t="s">
         <v>78</v>
       </c>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
-      <c r="L3" s="67"/>
+      <c r="J3" s="66"/>
+      <c r="K3" s="66"/>
+      <c r="L3" s="66"/>
       <c r="M3" t="s">
         <v>10</v>
       </c>

</xml_diff>